<commit_message>
Logo og følg tidsplan input
</commit_message>
<xml_diff>
--- a/AabenBane.xlsx
+++ b/AabenBane.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e885f104b2988143/AppUdvikling/AabenBaneHIK/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1abe8105c4474176/Active Supply/Programming/AabenBaneHIK/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EB8A371-DDAC-4368-B4D5-D33484B66C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{6EB8A371-DDAC-4368-B4D5-D33484B66C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBD39676-FC4B-4F10-8F39-5BBB4D09C2AC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tilmeldinger" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="41">
   <si>
     <t>Medlemsnr</t>
   </si>
@@ -82,9 +82,6 @@
     <t/>
   </si>
   <si>
-    <t>19:00;20:00;18:30;19:30</t>
-  </si>
-  <si>
     <t>13993</t>
   </si>
   <si>
@@ -143,6 +140,9 @@
   </si>
   <si>
     <t>Søren Schødt</t>
+  </si>
+  <si>
+    <t>19:00;20:00;18:30;19:30;20:30</t>
   </si>
 </sst>
 </file>
@@ -178,8 +178,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,13 +521,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.69921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -564,7 +565,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -595,19 +596,19 @@
       <c r="J2" t="s">
         <v>18</v>
       </c>
-      <c r="K2" t="s">
-        <v>19</v>
+      <c r="K2" s="1">
+        <v>0.85416666666666663</v>
       </c>
       <c r="L2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
       </c>
       <c r="C3">
         <v>4</v>
@@ -622,7 +623,7 @@
         <v>4</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H3" t="s">
         <v>17</v>
@@ -637,15 +638,15 @@
         <v>19</v>
       </c>
       <c r="L3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>26</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -660,7 +661,7 @@
         <v>2</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H4" t="s">
         <v>17</v>
@@ -675,15 +676,15 @@
         <v>19</v>
       </c>
       <c r="L4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>28</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -710,24 +711,24 @@
         <v>16</v>
       </c>
       <c r="K5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L5" t="s">
         <v>30</v>
       </c>
-      <c r="L5" t="s">
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>32</v>
-      </c>
-      <c r="B6" t="s">
-        <v>33</v>
       </c>
       <c r="C6">
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -754,12 +755,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s">
         <v>35</v>
-      </c>
-      <c r="B7" t="s">
-        <v>36</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -777,27 +778,27 @@
         <v>15</v>
       </c>
       <c r="H7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" t="s">
+        <v>19</v>
+      </c>
+      <c r="L7" t="s">
         <v>37</v>
       </c>
-      <c r="I7" t="s">
-        <v>19</v>
-      </c>
-      <c r="J7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" t="s">
-        <v>19</v>
-      </c>
-      <c r="L7" t="s">
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>39</v>
-      </c>
-      <c r="B8" t="s">
-        <v>40</v>
       </c>
       <c r="C8">
         <v>5</v>
@@ -812,7 +813,7 @@
         <v>4</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
         <v>17</v>
@@ -827,13 +828,13 @@
         <v>19</v>
       </c>
       <c r="L8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L8" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L1 A3:L8 A2:J2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>